<commit_message>
publish: fifteen history episodes premium, QA waived, landed in staging
accessDecision premium on all fifteen (AV, 2026-09-14), publishedAt stamped,
and audio + catalog rows upserted into lullable-staging.

QA was waived by AV without a device listen, on his explicit instruction —
recorded that way in every manifest's qa.deviceNotes rather than as a listen
that did not happen, the same wording used for Alexandria on 2026-08-20.

the-scriptorium-at-lindisfarne was verified 11/11 against the manifest in
staging. The other fourteen are uploaded and upserted but not yet verified,
so none of them can be promoted: production requires staging.verifiedAt and
the tool refuses without it.

Next: lullable.py verify <id> --env staging for the remaining fourteen, then
look at staging before any promote.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lullable_Story_Card_Tracker.xlsx
+++ b/Lullable_Story_Card_Tracker.xlsx
@@ -1378,17 +1378,17 @@
       <c r="B6" s="7" t="inlineStr"/>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="AC6" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD6" s="9" t="inlineStr">
@@ -1525,12 +1525,12 @@
       </c>
       <c r="AJ6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL6" s="9" t="inlineStr">
@@ -1560,12 +1560,12 @@
       </c>
       <c r="AQ6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS6" s="9" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="AT6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU6" s="9" t="inlineStr">
@@ -2549,17 +2549,17 @@
       <c r="B11" s="7" t="inlineStr"/>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="AC11" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD11" s="9" t="inlineStr">
@@ -2700,12 +2700,12 @@
       </c>
       <c r="AJ11" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK11" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL11" s="9" t="inlineStr">
@@ -2735,12 +2735,12 @@
       </c>
       <c r="AQ11" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR11" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS11" s="9" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="AT11" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU11" s="9" t="inlineStr">
@@ -3015,17 +3015,17 @@
       <c r="B13" s="7" t="inlineStr"/>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="AC13" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD13" s="9" t="inlineStr">
@@ -3162,12 +3162,12 @@
       </c>
       <c r="AJ13" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK13" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL13" s="9" t="inlineStr">
@@ -3197,12 +3197,12 @@
       </c>
       <c r="AQ13" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR13" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS13" s="9" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="AT13" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU13" s="9" t="inlineStr">
@@ -3240,17 +3240,17 @@
       <c r="B14" s="7" t="inlineStr"/>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -3286,7 +3286,7 @@
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="AC14" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD14" s="9" t="inlineStr">
@@ -3387,12 +3387,12 @@
       </c>
       <c r="AJ14" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK14" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL14" s="9" t="inlineStr">
@@ -3422,12 +3422,12 @@
       </c>
       <c r="AQ14" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR14" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS14" s="9" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="AT14" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU14" s="9" t="inlineStr">
@@ -3465,17 +3465,17 @@
       <c r="B15" s="7" t="inlineStr"/>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="AC15" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD15" s="9" t="inlineStr">
@@ -3616,12 +3616,12 @@
       </c>
       <c r="AJ15" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK15" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL15" s="9" t="inlineStr">
@@ -3651,12 +3651,12 @@
       </c>
       <c r="AQ15" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR15" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS15" s="9" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="AT15" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU15" s="9" t="inlineStr">
@@ -4640,17 +4640,17 @@
       <c r="B20" s="7" t="inlineStr"/>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
@@ -4690,7 +4690,7 @@
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="AC20" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD20" s="9" t="inlineStr">
@@ -4791,12 +4791,12 @@
       </c>
       <c r="AJ20" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK20" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL20" s="9" t="inlineStr">
@@ -4826,12 +4826,12 @@
       </c>
       <c r="AQ20" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR20" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS20" s="9" t="inlineStr">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="AT20" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU20" s="9" t="inlineStr">
@@ -5104,17 +5104,17 @@
       <c r="B22" s="7" t="inlineStr"/>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N22" s="7" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="AC22" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD22" s="9" t="inlineStr">
@@ -5255,12 +5255,12 @@
       </c>
       <c r="AJ22" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK22" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL22" s="9" t="inlineStr">
@@ -5290,12 +5290,12 @@
       </c>
       <c r="AQ22" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR22" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS22" s="9" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="AT22" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU22" s="9" t="inlineStr">
@@ -5333,17 +5333,17 @@
       <c r="B23" s="7" t="inlineStr"/>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="AC23" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD23" s="9" t="inlineStr">
@@ -5480,12 +5480,12 @@
       </c>
       <c r="AJ23" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK23" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL23" s="9" t="inlineStr">
@@ -5515,12 +5515,12 @@
       </c>
       <c r="AQ23" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR23" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS23" s="9" t="inlineStr">
@@ -5530,7 +5530,7 @@
       </c>
       <c r="AT23" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU23" s="9" t="inlineStr">
@@ -5558,17 +5558,17 @@
       <c r="B24" s="7" t="inlineStr"/>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N24" s="7" t="inlineStr">
@@ -5670,7 +5670,7 @@
       </c>
       <c r="AC24" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD24" s="9" t="inlineStr">
@@ -5705,12 +5705,12 @@
       </c>
       <c r="AJ24" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK24" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL24" s="9" t="inlineStr">
@@ -5740,12 +5740,12 @@
       </c>
       <c r="AQ24" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR24" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS24" s="9" t="inlineStr">
@@ -5755,7 +5755,7 @@
       </c>
       <c r="AT24" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU24" s="9" t="inlineStr">
@@ -6020,17 +6020,17 @@
       <c r="B26" s="7" t="inlineStr"/>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
@@ -6066,7 +6066,7 @@
       </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="AC26" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD26" s="9" t="inlineStr">
@@ -6167,12 +6167,12 @@
       </c>
       <c r="AJ26" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK26" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL26" s="9" t="inlineStr">
@@ -6202,12 +6202,12 @@
       </c>
       <c r="AQ26" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR26" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS26" s="9" t="inlineStr">
@@ -6217,7 +6217,7 @@
       </c>
       <c r="AT26" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU26" s="9" t="inlineStr">
@@ -8376,17 +8376,17 @@
       <c r="B36" s="7" t="inlineStr"/>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="M36" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N36" s="7" t="inlineStr">
@@ -8492,7 +8492,7 @@
       </c>
       <c r="AC36" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD36" s="9" t="inlineStr">
@@ -8527,12 +8527,12 @@
       </c>
       <c r="AJ36" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK36" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL36" s="9" t="inlineStr">
@@ -8562,12 +8562,12 @@
       </c>
       <c r="AQ36" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR36" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS36" s="9" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="AT36" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU36" s="9" t="inlineStr">
@@ -9079,17 +9079,17 @@
       <c r="B39" s="7" t="inlineStr"/>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
@@ -9129,7 +9129,7 @@
       </c>
       <c r="M39" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
@@ -9195,7 +9195,7 @@
       </c>
       <c r="AC39" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD39" s="9" t="inlineStr">
@@ -9230,12 +9230,12 @@
       </c>
       <c r="AJ39" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK39" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL39" s="9" t="inlineStr">
@@ -9265,12 +9265,12 @@
       </c>
       <c r="AQ39" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR39" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS39" s="9" t="inlineStr">
@@ -9280,7 +9280,7 @@
       </c>
       <c r="AT39" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU39" s="9" t="inlineStr">
@@ -9782,17 +9782,17 @@
       <c r="B42" s="7" t="inlineStr"/>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
@@ -9828,7 +9828,7 @@
       </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N42" s="7" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="AC42" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD42" s="9" t="inlineStr">
@@ -9929,12 +9929,12 @@
       </c>
       <c r="AJ42" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK42" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL42" s="9" t="inlineStr">
@@ -9964,12 +9964,12 @@
       </c>
       <c r="AQ42" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR42" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS42" s="9" t="inlineStr">
@@ -9979,7 +9979,7 @@
       </c>
       <c r="AT42" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU42" s="9" t="inlineStr">
@@ -10007,17 +10007,17 @@
       <c r="B43" s="7" t="inlineStr"/>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
@@ -10057,7 +10057,7 @@
       </c>
       <c r="M43" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr">
@@ -10123,7 +10123,7 @@
       </c>
       <c r="AC43" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD43" s="9" t="inlineStr">
@@ -10158,12 +10158,12 @@
       </c>
       <c r="AJ43" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK43" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL43" s="9" t="inlineStr">
@@ -10193,12 +10193,12 @@
       </c>
       <c r="AQ43" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR43" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS43" s="9" t="inlineStr">
@@ -10208,7 +10208,7 @@
       </c>
       <c r="AT43" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU43" s="9" t="inlineStr">
@@ -10473,17 +10473,17 @@
       <c r="B45" s="7" t="inlineStr"/>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>premium</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
@@ -10519,7 +10519,7 @@
       </c>
       <c r="M45" s="7" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2026-09-15T03:40:07Z</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr">
@@ -10585,7 +10585,7 @@
       </c>
       <c r="AC45" s="9" t="inlineStr">
         <is>
-          <t>rendered</t>
+          <t>staging</t>
         </is>
       </c>
       <c r="AD45" s="9" t="inlineStr">
@@ -10620,12 +10620,12 @@
       </c>
       <c r="AJ45" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AK45" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AL45" s="9" t="inlineStr">
@@ -10655,12 +10655,12 @@
       </c>
       <c r="AQ45" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AR45" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AS45" s="9" t="inlineStr">
@@ -10670,7 +10670,7 @@
       </c>
       <c r="AT45" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AU45" s="9" t="inlineStr">

</xml_diff>

<commit_message>
publish: fifteen history episodes promoted to production and verified
All fifteen promoted staging -> production and verified 11/11 each against
their manifests: title, access, publication state, active asset, bucket,
object path, byte size, sha256, asset status, duration, storage object.

Production catalogue is now 41 stories, all published, 38 premium.
Local: 42 stories, 41 PUBLISH READY, nothing stale.

These are live to users. QA was waived, not performed — nobody has listened
to the twelve hours this adds. Recorded that way in every manifest.

Open, noticed while querying and not investigated: production's
database_environment.apple_environment is 'sandbox' (updated 2026-09-14
17:54Z, not by this pipeline). Worth confirming it is intended now that new
premium content is live.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lullable_Story_Card_Tracker.xlsx
+++ b/Lullable_Story_Card_Tracker.xlsx
@@ -1378,7 +1378,7 @@
       <c r="B6" s="7" t="inlineStr"/>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -1490,12 +1490,12 @@
       </c>
       <c r="AC6" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD6" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE6" s="9" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="AV6" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW6" s="9" t="inlineStr">
@@ -2549,7 +2549,7 @@
       <c r="B11" s="7" t="inlineStr"/>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -2665,12 +2665,12 @@
       </c>
       <c r="AC11" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD11" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE11" s="9" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="AV11" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW11" s="9" t="inlineStr">
@@ -3015,7 +3015,7 @@
       <c r="B13" s="7" t="inlineStr"/>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -3127,12 +3127,12 @@
       </c>
       <c r="AC13" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD13" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE13" s="9" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="AV13" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW13" s="9" t="inlineStr">
@@ -3240,7 +3240,7 @@
       <c r="B14" s="7" t="inlineStr"/>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -3352,12 +3352,12 @@
       </c>
       <c r="AC14" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD14" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE14" s="9" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="AV14" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW14" s="9" t="inlineStr">
@@ -3465,7 +3465,7 @@
       <c r="B15" s="7" t="inlineStr"/>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -3581,12 +3581,12 @@
       </c>
       <c r="AC15" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD15" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE15" s="9" t="inlineStr">
@@ -3676,7 +3676,7 @@
       </c>
       <c r="AV15" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW15" s="9" t="inlineStr">
@@ -4640,7 +4640,7 @@
       <c r="B20" s="7" t="inlineStr"/>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -4756,12 +4756,12 @@
       </c>
       <c r="AC20" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD20" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE20" s="9" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="AV20" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW20" s="9" t="inlineStr">
@@ -5104,7 +5104,7 @@
       <c r="B22" s="7" t="inlineStr"/>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -5220,12 +5220,12 @@
       </c>
       <c r="AC22" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD22" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE22" s="9" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="AV22" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW22" s="9" t="inlineStr">
@@ -5333,7 +5333,7 @@
       <c r="B23" s="7" t="inlineStr"/>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -5445,12 +5445,12 @@
       </c>
       <c r="AC23" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD23" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE23" s="9" t="inlineStr">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="AV23" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW23" s="9" t="inlineStr">
@@ -5558,7 +5558,7 @@
       <c r="B24" s="7" t="inlineStr"/>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -5670,12 +5670,12 @@
       </c>
       <c r="AC24" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD24" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE24" s="9" t="inlineStr">
@@ -5765,7 +5765,7 @@
       </c>
       <c r="AV24" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW24" s="9" t="inlineStr">
@@ -6020,7 +6020,7 @@
       <c r="B26" s="7" t="inlineStr"/>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -6132,12 +6132,12 @@
       </c>
       <c r="AC26" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD26" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE26" s="9" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="AV26" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW26" s="9" t="inlineStr">
@@ -8376,7 +8376,7 @@
       <c r="B36" s="7" t="inlineStr"/>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -8492,12 +8492,12 @@
       </c>
       <c r="AC36" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD36" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE36" s="9" t="inlineStr">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="AV36" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW36" s="9" t="inlineStr">
@@ -9079,7 +9079,7 @@
       <c r="B39" s="7" t="inlineStr"/>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -9195,12 +9195,12 @@
       </c>
       <c r="AC39" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD39" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE39" s="9" t="inlineStr">
@@ -9290,7 +9290,7 @@
       </c>
       <c r="AV39" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW39" s="9" t="inlineStr">
@@ -9782,7 +9782,7 @@
       <c r="B42" s="7" t="inlineStr"/>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -9894,12 +9894,12 @@
       </c>
       <c r="AC42" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD42" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE42" s="9" t="inlineStr">
@@ -9989,7 +9989,7 @@
       </c>
       <c r="AV42" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW42" s="9" t="inlineStr">
@@ -10007,7 +10007,7 @@
       <c r="B43" s="7" t="inlineStr"/>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -10123,12 +10123,12 @@
       </c>
       <c r="AC43" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD43" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE43" s="9" t="inlineStr">
@@ -10218,7 +10218,7 @@
       </c>
       <c r="AV43" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW43" s="9" t="inlineStr">
@@ -10473,7 +10473,7 @@
       <c r="B45" s="7" t="inlineStr"/>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -10585,12 +10585,12 @@
       </c>
       <c r="AC45" s="9" t="inlineStr">
         <is>
-          <t>staging</t>
+          <t>published</t>
         </is>
       </c>
       <c r="AD45" s="9" t="inlineStr">
         <is>
-          <t>NOT READY</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="AE45" s="9" t="inlineStr">
@@ -10680,7 +10680,7 @@
       </c>
       <c r="AV45" s="9" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="AW45" s="9" t="inlineStr">

</xml_diff>